<commit_message>
Kit de Tareas Chocolatería (ES LIVE): 3 erratas de seguridad parcheadas en 7 celdas, sin cambio de versión
- Ganache de nata fresca y trufas de nata en frío a 0-4 °C (01 Apertura B25, 01 Cierre B6, 04 Dependiente B29,
  02 Moldeado B33) y con fecha de caducidad en 02 B31 (Reglamento UE 1169/2011, art. 24).
- 02 Moldeado B25: etiqueta con denominación, ingredientes con alérgenos destacados, peso neto, lote y fecha.
- 01 Apertura B10: quien tiene síntomas no entra en obrador ni mostrador (852/2004, anexo II, cap. VIII).
Parche en el XML de las celdas inlineStr (estilos, DV, CF y caché intactos; los otros 8 libros, mismo sha256);
volcado ES: solo esas 7 celdas; censo-entregables y gate-no-latinos del ES en 0. Mismos textos en el generador
y en el contenido v2.0. SPEC §5: erratas marcadas RESUELTAS.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Via: Claude Code
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/kit-tareas-chocolateria/01-apertura-cierre.xlsx
+++ b/astro-site/public/dl/kit-tareas-chocolateria/01-apertura-cierre.xlsx
@@ -908,7 +908,7 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Quien tenga vómitos, diarrea, fiebre o lesiones cutáneas infectadas NO manipula producto: comunicarlo al encargado y reasignar tarea</t>
+          <t>Quien tenga vómitos, diarrea, fiebre o lesiones cutáneas infectadas NO manipula producto ni entra en obrador ni mostrador: comunicarlo al encargado</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
@@ -1187,7 +1187,7 @@
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>Montar vitrina: bombones, tabletas, figuras, trufas</t>
+          <t>Montar vitrina: bombones, tabletas, figuras, trufas; los de ganache de nata fresca y las trufas de nata, solo en vitrina refrigerada a 0-4 °C</t>
         </is>
       </c>
       <c r="C25" s="15" t="inlineStr">
@@ -1587,7 +1587,7 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Retirar productos de vitrina y guardar en conservación</t>
+          <t>Retirar productos de vitrina y guardar en conservación; la ganache de nata fresca y las trufas de nata, a la cámara de 0-4 °C</t>
         </is>
       </c>
       <c r="C6" s="15" t="inlineStr">

</xml_diff>